<commit_message>
Show which part each treatment/cut service applies to
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019oxoH766RXuqLqXQEjeJHj
</commit_message>
<xml_diff>
--- a/Lista_de_materiais_04.01.3.000598_estilo_Nomus.xlsx
+++ b/Lista_de_materiais_04.01.3.000598_estilo_Nomus.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E188"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -444,6 +444,8 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,6 +474,16 @@
           <t>Código do componente</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Serviço aplicado em (peça)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Observação do serviço</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -692,6 +704,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>03.022-007308 - FLANGE</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -917,6 +939,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>03.022-007310 - CHAPA INFERIOR</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -992,6 +1024,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>03.022-007311 - CHAPA LATERAL</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1342,6 +1384,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>03.022-007355 - SUPORTE DO DISTRIBUIDOR</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1417,6 +1469,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>03.022-007326 - ANEL GUARDA PÓ</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1642,6 +1704,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>03.022-007365 - FLANGE DA TAMPA</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2067,6 +2139,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>03.022-007340 - PLACA CENTRAL</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2142,6 +2224,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>03.022-007332 - BUCHA DA PLACA CENTRAL</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2267,6 +2359,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>03.022-007336 - BUCHA CENTRAL 2</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2342,6 +2444,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>03.022-007335 - BUCHA CENTRAL</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Nitretação à gás (desenho 022-007335, nota 3)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2517,6 +2629,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>03.022-007343 - CHAPA DA ALAVANCA</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2592,6 +2714,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>03.022-007345 - BARRA SUPERIOR DA ALAVANCA</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2667,6 +2799,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>03.022-007350 - BARRA INFERIOR DA ALAVANCA</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2742,6 +2884,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>03.022-007351 - BUCHA DO CONJUNTO ALAVANCA</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2867,6 +3019,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>03.022-007338 - BASE DO SUPORTE</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2942,6 +3104,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>03.022-007339 - CHAPA DO SUPORTE</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3017,6 +3189,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>03.022-007353 - BUCHA MAIOR DO SUPORTE</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3092,6 +3274,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>03.022-007354 - BUCHA MENOR DO SUPORTE</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -3217,6 +3409,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>03.022-007357 - BUCHA DO BRAÇO ARTICULADO</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -3292,6 +3494,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>03.022-007356 - BRAÇO ARTICULADO</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -3417,6 +3629,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>03.022-007361 - ANEL DE AJUSTE MAIOR</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -3492,6 +3714,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>03.022-007364 - ANEL DE AJUSTE DO EIXO</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -3567,6 +3799,16 @@
           <t>09.1.0003</t>
         </is>
       </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>03.022-007360 - ANEL DE AJUSTE MENOR</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -3642,6 +3884,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>03.022-007358 - PINO MAIOR</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -3717,6 +3969,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>03.022-007363 - PINO MENOR DO BRAÇO</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -3792,6 +4054,16 @@
           <t>09.1.0002</t>
         </is>
       </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>03.022-007359 - PINO MENOR</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Nitretação em sais (nota do desenho da peça)</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -4215,6 +4487,16 @@
       <c r="E151" t="inlineStr">
         <is>
           <t>09.1.0003</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>03.022-007349 - BASE DO DISCO</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Chapa A516 / espessura fora da faixa de corte interno</t>
         </is>
       </c>
     </row>

</xml_diff>